<commit_message>
Fix BendingCoreService , Modify ServiceStartupViewModel ,Fix Bending publish issue.
</commit_message>
<xml_diff>
--- a/IPCSoftwares/IPCSoftware.App.Bending/Documents/Bending_Code_Docs.xlsx
+++ b/IPCSoftwares/IPCSoftware.App.Bending/Documents/Bending_Code_Docs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AOI DOCUMENT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IPCSOFTWARE_Refactoring\Vertex\IPCSoftwares\IPCSoftware.App.Bending\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="86">
   <si>
     <t>Sno</t>
   </si>
@@ -306,12 +306,97 @@
   <si>
     <t>In order to create new EventSource name , the Application/Visual Studio should run with Administrator previlages.</t>
   </si>
+  <si>
+    <t>For Background Core Service , user have to register Core Service as a "Window Service" as the following steps.</t>
+  </si>
+  <si>
+    <t>Open the Cmd Promt using Admin Rights and enter the following query-</t>
+  </si>
+  <si>
+    <r>
+      <t>sc create "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ServiceName</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" binpath="</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Path where Service .exe exist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" start=auto
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.499984740745262"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sc start "ServiceName"
+sc query "ServiceName"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;&gt;
+In case to delete  Registered Service-
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3" tint="0.499984740745262"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sc delete "ServiceName"</t>
+    </r>
+  </si>
+  <si>
+    <t>Tip - : Use ServiceName "IPCSoftware.CoreService.Bending" for Bending Service , "IPCSoftware.CoreService.AOI" for AOI service.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -370,6 +455,18 @@
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3" tint="0.499984740745262"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -662,6 +759,30 @@
       <alignment horizontal="left" indent="10"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -709,30 +830,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5924,142 +6021,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="55"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="42"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="43" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="58"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="61"/>
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="38"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2"/>
-      <c r="B5" s="53"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="55"/>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="B5" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="42"/>
+    </row>
+    <row r="6" spans="1:6" ht="91.2" customHeight="1">
       <c r="A6" s="2"/>
-      <c r="B6" s="53"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="55"/>
+      <c r="B6" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="38"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2"/>
-      <c r="B7" s="53"/>
-      <c r="C7" s="54"/>
-      <c r="D7" s="54"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="40" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="42"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2"/>
-      <c r="B8" s="53"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="55"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="42"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2"/>
-      <c r="B9" s="53"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="54"/>
-      <c r="F9" s="55"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="42"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2"/>
-      <c r="B10" s="53"/>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="55"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="42"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2"/>
-      <c r="B11" s="53"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="55"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2"/>
-      <c r="B12" s="53"/>
-      <c r="C12" s="54"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="54"/>
-      <c r="F12" s="55"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="42"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2"/>
-      <c r="B13" s="53"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
-      <c r="E13" s="54"/>
-      <c r="F13" s="55"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="42"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2"/>
-      <c r="B14" s="53"/>
-      <c r="C14" s="54"/>
-      <c r="D14" s="54"/>
-      <c r="E14" s="54"/>
-      <c r="F14" s="55"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="41"/>
+      <c r="F14" s="42"/>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2"/>
-      <c r="B15" s="53"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="55"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="41"/>
+      <c r="F15" s="42"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2"/>
-      <c r="B16" s="53"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="55"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -6073,14 +6180,15 @@
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B6:F6"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6097,17 +6205,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="45" t="s">
+      <c r="B1" s="53"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="10" t="s">
@@ -6164,11 +6272,11 @@
       <c r="C4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="F4" s="39" t="s">
+      <c r="E4" s="46"/>
+      <c r="F4" s="49" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="8"/>
@@ -6184,9 +6292,9 @@
       <c r="C5" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="40"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="50"/>
       <c r="G5" s="8"/>
       <c r="H5" s="5"/>
     </row>
@@ -6200,9 +6308,9 @@
       <c r="C6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="40"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="50"/>
       <c r="G6" s="8"/>
       <c r="H6" s="5"/>
     </row>
@@ -6216,9 +6324,9 @@
       <c r="C7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="38"/>
-      <c r="E7" s="38"/>
-      <c r="F7" s="41"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="51"/>
       <c r="G7" s="8"/>
       <c r="H7" s="5"/>
     </row>
@@ -6329,13 +6437,13 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="47"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48"/>
-      <c r="G13" s="49"/>
+      <c r="A13" s="57"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="59"/>
     </row>
     <row r="14" spans="1:8" ht="27.6">
       <c r="A14" s="7">
@@ -6584,24 +6692,24 @@
   <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="4" spans="3:9">
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
+      <c r="D4" s="60"/>
+      <c r="E4" s="60"/>
+      <c r="F4" s="60"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="60"/>
+      <c r="I4" s="60"/>
     </row>
     <row r="5" spans="3:9">
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
+      <c r="C5" s="60"/>
+      <c r="D5" s="60"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="60"/>
+      <c r="G5" s="60"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="60"/>
     </row>
     <row r="8" spans="3:9">
       <c r="H8" t="s">
@@ -6624,18 +6732,18 @@
       </c>
     </row>
     <row r="40" spans="2:11">
-      <c r="B40" s="50" t="s">
+      <c r="B40" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="C40" s="50"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="50"/>
-      <c r="H40" s="50"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="50"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="60"/>
+      <c r="E40" s="60"/>
+      <c r="F40" s="60"/>
+      <c r="G40" s="60"/>
+      <c r="H40" s="60"/>
+      <c r="I40" s="60"/>
+      <c r="J40" s="60"/>
+      <c r="K40" s="60"/>
     </row>
     <row r="43" spans="2:11">
       <c r="H43" t="s">
@@ -6658,18 +6766,18 @@
       </c>
     </row>
     <row r="59" spans="2:12">
-      <c r="B59" s="50" t="s">
+      <c r="B59" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="50"/>
-      <c r="D59" s="50"/>
-      <c r="E59" s="50"/>
-      <c r="F59" s="50"/>
-      <c r="G59" s="50"/>
-      <c r="H59" s="50"/>
-      <c r="I59" s="50"/>
-      <c r="J59" s="50"/>
-      <c r="K59" s="50"/>
+      <c r="C59" s="60"/>
+      <c r="D59" s="60"/>
+      <c r="E59" s="60"/>
+      <c r="F59" s="60"/>
+      <c r="G59" s="60"/>
+      <c r="H59" s="60"/>
+      <c r="I59" s="60"/>
+      <c r="J59" s="60"/>
+      <c r="K59" s="60"/>
     </row>
     <row r="62" spans="2:12">
       <c r="L62" t="s">
@@ -6714,18 +6822,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="7:17">
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="50" t="s">
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
     </row>
     <row r="6" spans="7:17" ht="15.6">
       <c r="P6" s="31" t="s">

</xml_diff>

<commit_message>
Removal of HardCoded Data Phase1
</commit_message>
<xml_diff>
--- a/IPCSoftwares/IPCSoftware.App.Bending/Documents/Bending_Code_Docs.xlsx
+++ b/IPCSoftwares/IPCSoftware.App.Bending/Documents/Bending_Code_Docs.xlsx
@@ -9,14 +9,15 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9384" tabRatio="689"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9384" tabRatio="689" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="BendingCodeDocs" sheetId="15" r:id="rId1"/>
-    <sheet name="Code_Optimize" sheetId="4" r:id="rId2"/>
-    <sheet name="DeviceConfig-Optimize" sheetId="6" r:id="rId3"/>
-    <sheet name="TraceLog CallRef" sheetId="7" r:id="rId4"/>
-    <sheet name="ErrorLogging-Struct" sheetId="12" r:id="rId5"/>
+    <sheet name="Remove HardCode Data" sheetId="16" r:id="rId2"/>
+    <sheet name="Code_Optimize" sheetId="4" r:id="rId3"/>
+    <sheet name="DeviceConfig-Optimize" sheetId="6" r:id="rId4"/>
+    <sheet name="TraceLog CallRef" sheetId="7" r:id="rId5"/>
+    <sheet name="ErrorLogging-Struct" sheetId="12" r:id="rId6"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="119">
   <si>
     <t>Sno</t>
   </si>
@@ -390,6 +391,105 @@
   </si>
   <si>
     <t>Tip - : Use ServiceName "IPCSoftware.CoreService.Bending" for Bending Service , "IPCSoftware.CoreService.AOI" for AOI service.</t>
+  </si>
+  <si>
+    <t>NameScape</t>
+  </si>
+  <si>
+    <t>FileName</t>
+  </si>
+  <si>
+    <t>MethodUsed</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>IPCSoftware.App.ViewModels</t>
+  </si>
+  <si>
+    <t>OEEDashboardViewModel</t>
+  </si>
+  <si>
+    <t>ToggleMacMini()</t>
+  </si>
+  <si>
+    <t>IsMacMiniEnabled</t>
+  </si>
+  <si>
+    <t>Line No.</t>
+  </si>
+  <si>
+    <t>485-486</t>
+  </si>
+  <si>
+    <t>InspectionXUnit, InspectionYUnit, InspectionAngleUnit</t>
+  </si>
+  <si>
+    <t>AeLimitViewModel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SaveAndTransferAsync()</t>
+  </si>
+  <si>
+    <t>146-151</t>
+  </si>
+  <si>
+    <t>IPCSoftware.UI.CommonViews.ViewModels</t>
+  </si>
+  <si>
+    <t>143-148</t>
+  </si>
+  <si>
+    <t>Protocol, MacMiniIpAddress, Port, EndPoint, PreviousMachineCode, AOIMachineCode</t>
+  </si>
+  <si>
+    <t>205-209</t>
+  </si>
+  <si>
+    <t>SaveSettings()</t>
+  </si>
+  <si>
+    <t>ApiTestViewModel</t>
+  </si>
+  <si>
+    <t>Tightly couple binding - UI - CoreService</t>
+  </si>
+  <si>
+    <t>Present dependency pattern</t>
+  </si>
+  <si>
+    <t>Start Date- 13/05/2026</t>
+  </si>
+  <si>
+    <t>Complete Date -</t>
+  </si>
+  <si>
+    <t>Depedency File</t>
+  </si>
+  <si>
+    <t>appSettings.json</t>
+  </si>
+  <si>
+    <t>// Instead of:</t>
+  </si>
+  <si>
+    <t>File.WriteAllText(appSettingsPath, jsonObj.ToString());</t>
+  </si>
+  <si>
+    <t>// Use:</t>
+  </si>
+  <si>
+    <t>await _coreClient.WriteSettingAsync("External.IsMacMiniEnabled", newValue);</t>
+  </si>
+  <si>
+    <t>💡 Proposed Solution Pattern</t>
+  </si>
+  <si>
+    <t>Replace file writes with TCP Request/Response:</t>
+  </si>
+  <si>
+    <t>Proposed</t>
   </si>
 </sst>
 </file>
@@ -666,7 +766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -759,6 +859,29 @@
       <alignment horizontal="left" indent="10"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -771,9 +894,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -782,6 +902,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -825,9 +951,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -849,6 +972,784 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1051560</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>815340</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="13" name="Group 12"/>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="2392680" y="4114800"/>
+          <a:ext cx="8039100" cy="2240280"/>
+          <a:chOff x="2392680" y="4114800"/>
+          <a:chExt cx="5882640" cy="2240280"/>
+        </a:xfrm>
+        <a:effectLst>
+          <a:outerShdw blurRad="50800" dist="38100" dir="8100000" algn="tr" rotWithShape="0">
+            <a:prstClr val="black">
+              <a:alpha val="40000"/>
+            </a:prstClr>
+          </a:outerShdw>
+        </a:effectLst>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="Rounded Rectangle 1"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2392680" y="4168140"/>
+            <a:ext cx="1920240" cy="617220"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent2">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent2"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent2"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>UI LAYER </a:t>
+            </a:r>
+            <a:br>
+              <a:rPr lang="en-US" sz="1100"/>
+            </a:br>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>VIEW MODEL</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="Rounded Rectangle 2"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6225540" y="4130040"/>
+            <a:ext cx="1920240" cy="617220"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent2">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent2"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent2"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>appSettings.json</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="4" name="Rounded Rectangle 3"/>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6355080" y="5737860"/>
+            <a:ext cx="1920240" cy="617220"/>
+          </a:xfrm>
+          <a:prstGeom prst="roundRect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent2">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent2"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent2"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Core Service</a:t>
+            </a:r>
+            <a:br>
+              <a:rPr lang="en-US" sz="1100"/>
+            </a:br>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>(Background)</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="7" name="Straight Arrow Connector 6"/>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipV="1">
+            <a:off x="4549140" y="4472940"/>
+            <a:ext cx="1577340" cy="0"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="8" name="Straight Arrow Connector 7"/>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6995160" y="4846320"/>
+            <a:ext cx="0" cy="754380"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="TextBox 10"/>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7018020" y="5029200"/>
+            <a:ext cx="1043940" cy="365760"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-US" sz="900">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>IOption&lt;T&gt;</a:t>
+            </a:r>
+            <a:br>
+              <a:rPr lang="en-US" sz="900">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+            </a:br>
+            <a:r>
+              <a:rPr lang="en-US" sz="900">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>(Reload</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="900" baseline="0">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t> Delay)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="900">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="TextBox 11"/>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="4488180" y="4114800"/>
+            <a:ext cx="1699260" cy="220980"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" smtClean="0">
+                <a:solidFill>
+                  <a:schemeClr val="dk1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>File.WriteAllText </a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="900">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1295400</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3919562</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Rounded Rectangle 13"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2636520" y="8214360"/>
+          <a:ext cx="2624162" cy="617220"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent2">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>UI LAYER </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>VIEW MODEL</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>88558</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1059180</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="Rounded Rectangle 15"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8051458" y="9784080"/>
+          <a:ext cx="2624162" cy="617220"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent2">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>Core Service</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>(Background)</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3630279</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1516380</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="18" name="Straight Arrow Connector 17"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4971399" y="9174480"/>
+          <a:ext cx="2793381" cy="1226820"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>4107180</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="21" name="Straight Arrow Connector 20"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="5448300" y="8488680"/>
+          <a:ext cx="2697480" cy="1196340"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1127760</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="TextBox 22"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6377940" y="8709660"/>
+          <a:ext cx="2712720" cy="289560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Response</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> PAckage  (new ID 9)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="900">
+            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3589020</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1003915</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="TextBox 23"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4930140" y="9867900"/>
+          <a:ext cx="2322175" cy="220980"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" smtClean="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Request Package</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="900">
+            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2712720</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>108248</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="944880" y="11003280"/>
+          <a:ext cx="3108960" cy="2074208"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -3635,7 +4536,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -5527,7 +6428,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -6021,155 +6922,161 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="52" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="42"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="48"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="44"/>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="55"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="38"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="51"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2"/>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="42"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="48"/>
     </row>
     <row r="6" spans="1:6" ht="91.2" customHeight="1">
       <c r="A6" s="2"/>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="38"/>
+      <c r="C6" s="50"/>
+      <c r="D6" s="50"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="51"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2"/>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="46" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="42"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="48"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="42"/>
+      <c r="B8" s="46"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="48"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="41"/>
-      <c r="F9" s="42"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="48"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2"/>
-      <c r="B10" s="40"/>
-      <c r="C10" s="41"/>
-      <c r="D10" s="41"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="42"/>
+      <c r="B10" s="46"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="48"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2"/>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="41"/>
-      <c r="F11" s="42"/>
+      <c r="B11" s="46"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="47"/>
+      <c r="F11" s="48"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2"/>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="42"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="48"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2"/>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="41"/>
-      <c r="F13" s="42"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="47"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="48"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="42"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="48"/>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2"/>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="42"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="47"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="48"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2"/>
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="42"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B15:F15"/>
@@ -6180,12 +7087,6 @@
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6193,6 +7094,288 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:H215"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
+  <cols>
+    <col min="3" max="3" width="64.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" customWidth="1"/>
+    <col min="7" max="7" width="44.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.69921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8">
+      <c r="B1" s="57" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="57"/>
+    </row>
+    <row r="2" spans="2:8">
+      <c r="B2" s="56" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="44"/>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="F3" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" s="42" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4" s="36">
+        <v>1</v>
+      </c>
+      <c r="C4" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" s="43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5" s="36">
+        <v>2</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6" s="36">
+        <v>3</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H6" s="43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="27.6">
+      <c r="B7" s="38">
+        <v>4</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="H7" s="43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8" s="36"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9" s="36"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10" s="36"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11" s="36"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12" s="36"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13" s="36"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14" s="36"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15" s="36"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16" s="36"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" s="41" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="3:3">
+      <c r="C44" s="41" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="208" spans="3:3">
+      <c r="C208" s="41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="210" spans="3:3">
+      <c r="C210" s="45" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="211" spans="3:3">
+      <c r="C211" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="212" spans="3:3">
+      <c r="C212" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="214" spans="3:3">
+      <c r="C214" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="215" spans="3:3">
+      <c r="C215" t="s">
+        <v>115</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
@@ -6205,17 +7388,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="55" t="s">
+      <c r="B1" s="65"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="67" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="10" t="s">
@@ -6272,11 +7455,11 @@
       <c r="C4" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="49" t="s">
+      <c r="E4" s="58"/>
+      <c r="F4" s="61" t="s">
         <v>5</v>
       </c>
       <c r="G4" s="8"/>
@@ -6292,9 +7475,9 @@
       <c r="C5" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="50"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="62"/>
       <c r="G5" s="8"/>
       <c r="H5" s="5"/>
     </row>
@@ -6308,9 +7491,9 @@
       <c r="C6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="50"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="8"/>
       <c r="H6" s="5"/>
     </row>
@@ -6324,9 +7507,9 @@
       <c r="C7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="51"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="63"/>
       <c r="G7" s="8"/>
       <c r="H7" s="5"/>
     </row>
@@ -6437,13 +7620,13 @@
       <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="57"/>
-      <c r="B13" s="58"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="58"/>
-      <c r="E13" s="58"/>
-      <c r="F13" s="58"/>
-      <c r="G13" s="59"/>
+      <c r="A13" s="69"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
+      <c r="G13" s="71"/>
     </row>
     <row r="14" spans="1:8" ht="27.6">
       <c r="A14" s="7">
@@ -6686,30 +7869,30 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B4:L73"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData>
     <row r="4" spans="3:9">
-      <c r="C4" s="60" t="s">
+      <c r="C4" s="57" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="60"/>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
     </row>
     <row r="5" spans="3:9">
-      <c r="C5" s="60"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
-      <c r="F5" s="60"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="60"/>
-      <c r="I5" s="60"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57"/>
+      <c r="F5" s="57"/>
+      <c r="G5" s="57"/>
+      <c r="H5" s="57"/>
+      <c r="I5" s="57"/>
     </row>
     <row r="8" spans="3:9">
       <c r="H8" t="s">
@@ -6732,18 +7915,18 @@
       </c>
     </row>
     <row r="40" spans="2:11">
-      <c r="B40" s="60" t="s">
+      <c r="B40" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="60"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="60"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="57"/>
+      <c r="E40" s="57"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="57"/>
+      <c r="I40" s="57"/>
+      <c r="J40" s="57"/>
+      <c r="K40" s="57"/>
     </row>
     <row r="43" spans="2:11">
       <c r="H43" t="s">
@@ -6766,18 +7949,18 @@
       </c>
     </row>
     <row r="59" spans="2:12">
-      <c r="B59" s="60" t="s">
+      <c r="B59" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="C59" s="60"/>
-      <c r="D59" s="60"/>
-      <c r="E59" s="60"/>
-      <c r="F59" s="60"/>
-      <c r="G59" s="60"/>
-      <c r="H59" s="60"/>
-      <c r="I59" s="60"/>
-      <c r="J59" s="60"/>
-      <c r="K59" s="60"/>
+      <c r="C59" s="57"/>
+      <c r="D59" s="57"/>
+      <c r="E59" s="57"/>
+      <c r="F59" s="57"/>
+      <c r="G59" s="57"/>
+      <c r="H59" s="57"/>
+      <c r="I59" s="57"/>
+      <c r="J59" s="57"/>
+      <c r="K59" s="57"/>
     </row>
     <row r="62" spans="2:12">
       <c r="L62" t="s">
@@ -6810,7 +7993,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="G1:R33"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
@@ -6822,18 +8005,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="7:17">
-      <c r="G1" s="61" t="s">
+      <c r="G1" s="72" t="s">
         <v>70</v>
       </c>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
-      <c r="L1" s="60" t="s">
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
+      <c r="J1" s="72"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="57" t="s">
         <v>77</v>
       </c>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
+      <c r="M1" s="57"/>
+      <c r="N1" s="57"/>
     </row>
     <row r="6" spans="7:17" ht="15.6">
       <c r="P6" s="31" t="s">
@@ -6930,7 +8113,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A71"/>
   <sheetFormatPr defaultRowHeight="13.8"/>

</xml_diff>